<commit_message>
sync: 1 file(s) changed — 2026-09-05 19:58
</commit_message>
<xml_diff>
--- a/outputs/inc42/inc42-icp-and-role-definition.xlsx
+++ b/outputs/inc42/inc42-icp-and-role-definition.xlsx
@@ -9628,7 +9628,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Across 49 distinct values in 5 formats.</t>
+          <t>Across 50 distinct values in 5 formats.</t>
         </is>
       </c>
     </row>
@@ -9728,7 +9728,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  = usable AND in-market</t>
+          <t>Usable AND in-market (net)</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -12823,7 +12823,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>49 distinct values on Media, 40 on DataLabs, for roughly 11 real concepts.</t>
+          <t>50 distinct values on Media, 40 on DataLabs, for roughly 11 real concepts.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">

</xml_diff>